<commit_message>
Fix price updater - now fetching live prices correctly
</commit_message>
<xml_diff>
--- a/Funfamily_Stock_Tracker.xlsx
+++ b/Funfamily_Stock_Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deposit Sheet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Sheet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Deposit Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Stock Sheet" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,10 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="166" formatCode="DD/MM/YYYY"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -65,7 +64,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -73,12 +72,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -535,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -559,7 +560,7 @@
           <t>Current Date</t>
         </is>
       </c>
-      <c r="B1" s="5" t="n">
+      <c r="B1" s="9" t="n">
         <v>46095</v>
       </c>
     </row>
@@ -636,7 +637,7 @@
           <t>Shawn Mun</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n">
+      <c r="B3" s="10" t="n">
         <v>45614</v>
       </c>
       <c r="C3" s="2" t="n">
@@ -674,13 +675,13 @@
         <v>15.7252</v>
       </c>
       <c r="K3" s="8" t="n">
-        <v>17.38</v>
+        <v>17.034</v>
       </c>
       <c r="L3" s="8" t="n">
-        <v>5526.161829</v>
+        <v>5416.147457</v>
       </c>
       <c r="M3" s="8" t="n">
-        <v>526.161829</v>
+        <v>416.147457</v>
       </c>
     </row>
     <row r="4">
@@ -689,7 +690,7 @@
           <t>Shawn Mun</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n">
+      <c r="B4" s="10" t="n">
         <v>46020</v>
       </c>
       <c r="C4" s="2" t="n">
@@ -727,13 +728,13 @@
         <v>17.7045</v>
       </c>
       <c r="K4" s="8" t="n">
-        <v>17.38</v>
+        <v>17.034</v>
       </c>
       <c r="L4" s="8" t="n">
-        <v>9816.713265</v>
+        <v>9621.282949</v>
       </c>
       <c r="M4" s="8" t="n">
-        <v>-183.286735</v>
+        <v>-378.717051</v>
       </c>
     </row>
     <row r="5">
@@ -742,7 +743,7 @@
           <t>Shawn Mun</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="10" t="n">
         <v>46043</v>
       </c>
       <c r="C5" s="2" t="n">
@@ -780,13 +781,13 @@
         <v>17.5844</v>
       </c>
       <c r="K5" s="8" t="n">
-        <v>17.38</v>
+        <v>17.034</v>
       </c>
       <c r="L5" s="8" t="n">
-        <v>4941.880303</v>
+        <v>4843.497758</v>
       </c>
       <c r="M5" s="8" t="n">
-        <v>-58.119697</v>
+        <v>-156.502242</v>
       </c>
     </row>
     <row r="6">
@@ -795,7 +796,7 @@
           <t>Jasmine</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="10" t="n">
         <v>45912</v>
       </c>
       <c r="C6" s="2" t="n">
@@ -833,13 +834,13 @@
         <v>17.7186</v>
       </c>
       <c r="K6" s="8" t="n">
-        <v>17.38</v>
+        <v>17.034</v>
       </c>
       <c r="L6" s="8" t="n">
-        <v>4512.094635</v>
+        <v>4422.268228</v>
       </c>
       <c r="M6" s="8" t="n">
-        <v>-87.905365</v>
+        <v>-177.731772</v>
       </c>
     </row>
     <row r="7">
@@ -848,7 +849,7 @@
           <t>Jasmine</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="10" t="n">
         <v>46058</v>
       </c>
       <c r="C7" s="2" t="n">
@@ -886,13 +887,13 @@
         <v>322.79</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>370.6</v>
+        <v>338.31</v>
       </c>
       <c r="L7" s="8" t="n">
-        <v>5850.655621</v>
+        <v>5340.893926</v>
       </c>
       <c r="M7" s="8" t="n">
-        <v>754.775621</v>
+        <v>245.013926</v>
       </c>
     </row>
     <row r="8">
@@ -901,7 +902,7 @@
           <t>Jasmine</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="10" t="n">
         <v>46076</v>
       </c>
       <c r="C8" s="2" t="n">
@@ -939,15 +940,16 @@
         <v>393.48</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>394.16</v>
+        <v>395.55</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>10017.28169</v>
+        <v>10052.607192</v>
       </c>
       <c r="M8" s="8" t="n">
-        <v>17.281692</v>
-      </c>
-    </row>
+        <v>52.607192</v>
+      </c>
+    </row>
+    <row r="9"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Amended how the calculation for Add stock is done and also added a new function called remove stock.
</commit_message>
<xml_diff>
--- a/Funfamily_Stock_Tracker.xlsx
+++ b/Funfamily_Stock_Tracker.xlsx
@@ -17,9 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -64,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -80,6 +81,7 @@
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -949,7 +951,39 @@
         <v>52.607192</v>
       </c>
     </row>
-    <row r="9"/>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Jasmine</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>46096</v>
+      </c>
+      <c r="C9" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>IBKR</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>